<commit_message>
mejora en la invitaión personalizada
</commit_message>
<xml_diff>
--- a/Generador de invitaciones.xlsx
+++ b/Generador de invitaciones.xlsx
@@ -445,15 +445,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,6 +467,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -481,20 +481,15 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Firma / nota (opcional)</t>
+          <t>Cupos (número)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Cupos (número)</t>
+          <t>Invitados (nombres separados por coma)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Invitados (nombres separados por coma)</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>URL generada</t>
         </is>
@@ -511,17 +506,11 @@
           <t>Adela Parrales</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="C4" t="n">
         <v>1</v>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" s="2">
-        <f>$B$1&amp;"?titulo="&amp;ENCODEURL(A4)&amp;"&amp;invitado="&amp;ENCODEURL(B4)&amp;IF(C4&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C4),"")&amp;"&amp;admision="&amp;ENCODEURL(D4&amp;" persona"&amp;IF(D4=1,"","s"))&amp;IF(E4&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E4),"")</f>
+      <c r="E4" s="2">
+        <f>$B$1&amp;"?titulo="&amp;ENCODEURL(A4)&amp;"&amp;invitado="&amp;ENCODEURL(B4)&amp;"&amp;admision="&amp;ENCODEURL(C4&amp;" persona"&amp;IF(C4=1,"","s"))&amp;IF(D4&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D4),"")</f>
         <v/>
       </c>
     </row>
@@ -536,17 +525,16 @@
           <t>Familia Parrales</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="n">
+      <c r="C5" t="n">
         <v>3</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Adela Parrales, Juan Parrales, María Parrales</t>
         </is>
       </c>
-      <c r="F5" s="2">
-        <f>$B$1&amp;"?titulo="&amp;ENCODEURL(A5)&amp;"&amp;invitado="&amp;ENCODEURL(B5)&amp;IF(C5&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C5),"")&amp;"&amp;admision="&amp;ENCODEURL(D5&amp;" persona"&amp;IF(D5=1,"","s"))&amp;IF(E5&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E5),"")</f>
+      <c r="E5" s="2">
+        <f>$B$1&amp;"?titulo="&amp;ENCODEURL(A5)&amp;"&amp;invitado="&amp;ENCODEURL(B5)&amp;"&amp;admision="&amp;ENCODEURL(C5&amp;" persona"&amp;IF(C5=1,"","s"))&amp;IF(D5&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D5),"")</f>
         <v/>
       </c>
     </row>
@@ -561,201 +549,196 @@
           <t>Luis y Carmen Vera</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Con cariño</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+      <c r="C6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Luis Vera, Carmen Vera</t>
         </is>
       </c>
-      <c r="F6" s="2">
-        <f>$B$1&amp;"?titulo="&amp;ENCODEURL(A6)&amp;"&amp;invitado="&amp;ENCODEURL(B6)&amp;IF(C6&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C6),"")&amp;"&amp;admision="&amp;ENCODEURL(D6&amp;" persona"&amp;IF(D6=1,"","s"))&amp;IF(E6&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E6),"")</f>
+      <c r="E6" s="2">
+        <f>$B$1&amp;"?titulo="&amp;ENCODEURL(A6)&amp;"&amp;invitado="&amp;ENCODEURL(B6)&amp;"&amp;admision="&amp;ENCODEURL(C6&amp;" persona"&amp;IF(C6=1,"","s"))&amp;IF(D6&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D6),"")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="F7" s="2">
-        <f>IF(B7="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A7)&amp;"&amp;invitado="&amp;ENCODEURL(B7)&amp;IF(C7&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C7),"")&amp;"&amp;admision="&amp;ENCODEURL(D7&amp;" persona"&amp;IF(D7=1,"","s"))&amp;IF(E7&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E7),""))</f>
+      <c r="E7" s="2">
+        <f>IF(B7="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A7)&amp;"&amp;invitado="&amp;ENCODEURL(B7)&amp;"&amp;admision="&amp;ENCODEURL(C7&amp;" persona"&amp;IF(C7=1,"","s"))&amp;IF(D7&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D7),""))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="F8" s="2">
-        <f>IF(B8="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A8)&amp;"&amp;invitado="&amp;ENCODEURL(B8)&amp;IF(C8&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C8),"")&amp;"&amp;admision="&amp;ENCODEURL(D8&amp;" persona"&amp;IF(D8=1,"","s"))&amp;IF(E8&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E8),""))</f>
+      <c r="E8" s="2">
+        <f>IF(B8="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A8)&amp;"&amp;invitado="&amp;ENCODEURL(B8)&amp;"&amp;admision="&amp;ENCODEURL(C8&amp;" persona"&amp;IF(C8=1,"","s"))&amp;IF(D8&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D8),""))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="F9" s="2">
-        <f>IF(B9="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A9)&amp;"&amp;invitado="&amp;ENCODEURL(B9)&amp;IF(C9&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C9),"")&amp;"&amp;admision="&amp;ENCODEURL(D9&amp;" persona"&amp;IF(D9=1,"","s"))&amp;IF(E9&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E9),""))</f>
+      <c r="E9" s="2">
+        <f>IF(B9="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A9)&amp;"&amp;invitado="&amp;ENCODEURL(B9)&amp;"&amp;admision="&amp;ENCODEURL(C9&amp;" persona"&amp;IF(C9=1,"","s"))&amp;IF(D9&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D9),""))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="F10" s="2">
-        <f>IF(B10="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A10)&amp;"&amp;invitado="&amp;ENCODEURL(B10)&amp;IF(C10&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C10),"")&amp;"&amp;admision="&amp;ENCODEURL(D10&amp;" persona"&amp;IF(D10=1,"","s"))&amp;IF(E10&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E10),""))</f>
+      <c r="E10" s="2">
+        <f>IF(B10="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A10)&amp;"&amp;invitado="&amp;ENCODEURL(B10)&amp;"&amp;admision="&amp;ENCODEURL(C10&amp;" persona"&amp;IF(C10=1,"","s"))&amp;IF(D10&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D10),""))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="F11" s="2">
-        <f>IF(B11="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A11)&amp;"&amp;invitado="&amp;ENCODEURL(B11)&amp;IF(C11&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C11),"")&amp;"&amp;admision="&amp;ENCODEURL(D11&amp;" persona"&amp;IF(D11=1,"","s"))&amp;IF(E11&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E11),""))</f>
+      <c r="E11" s="2">
+        <f>IF(B11="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A11)&amp;"&amp;invitado="&amp;ENCODEURL(B11)&amp;"&amp;admision="&amp;ENCODEURL(C11&amp;" persona"&amp;IF(C11=1,"","s"))&amp;IF(D11&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D11),""))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="F12" s="2">
-        <f>IF(B12="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A12)&amp;"&amp;invitado="&amp;ENCODEURL(B12)&amp;IF(C12&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C12),"")&amp;"&amp;admision="&amp;ENCODEURL(D12&amp;" persona"&amp;IF(D12=1,"","s"))&amp;IF(E12&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E12),""))</f>
+      <c r="E12" s="2">
+        <f>IF(B12="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A12)&amp;"&amp;invitado="&amp;ENCODEURL(B12)&amp;"&amp;admision="&amp;ENCODEURL(C12&amp;" persona"&amp;IF(C12=1,"","s"))&amp;IF(D12&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D12),""))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="F13" s="2">
-        <f>IF(B13="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A13)&amp;"&amp;invitado="&amp;ENCODEURL(B13)&amp;IF(C13&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C13),"")&amp;"&amp;admision="&amp;ENCODEURL(D13&amp;" persona"&amp;IF(D13=1,"","s"))&amp;IF(E13&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E13),""))</f>
+      <c r="E13" s="2">
+        <f>IF(B13="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A13)&amp;"&amp;invitado="&amp;ENCODEURL(B13)&amp;"&amp;admision="&amp;ENCODEURL(C13&amp;" persona"&amp;IF(C13=1,"","s"))&amp;IF(D13&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D13),""))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="F14" s="2">
-        <f>IF(B14="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A14)&amp;"&amp;invitado="&amp;ENCODEURL(B14)&amp;IF(C14&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C14),"")&amp;"&amp;admision="&amp;ENCODEURL(D14&amp;" persona"&amp;IF(D14=1,"","s"))&amp;IF(E14&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E14),""))</f>
+      <c r="E14" s="2">
+        <f>IF(B14="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A14)&amp;"&amp;invitado="&amp;ENCODEURL(B14)&amp;"&amp;admision="&amp;ENCODEURL(C14&amp;" persona"&amp;IF(C14=1,"","s"))&amp;IF(D14&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D14),""))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="F15" s="2">
-        <f>IF(B15="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A15)&amp;"&amp;invitado="&amp;ENCODEURL(B15)&amp;IF(C15&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C15),"")&amp;"&amp;admision="&amp;ENCODEURL(D15&amp;" persona"&amp;IF(D15=1,"","s"))&amp;IF(E15&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E15),""))</f>
+      <c r="E15" s="2">
+        <f>IF(B15="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A15)&amp;"&amp;invitado="&amp;ENCODEURL(B15)&amp;"&amp;admision="&amp;ENCODEURL(C15&amp;" persona"&amp;IF(C15=1,"","s"))&amp;IF(D15&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D15),""))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="F16" s="2">
-        <f>IF(B16="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A16)&amp;"&amp;invitado="&amp;ENCODEURL(B16)&amp;IF(C16&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C16),"")&amp;"&amp;admision="&amp;ENCODEURL(D16&amp;" persona"&amp;IF(D16=1,"","s"))&amp;IF(E16&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E16),""))</f>
+      <c r="E16" s="2">
+        <f>IF(B16="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A16)&amp;"&amp;invitado="&amp;ENCODEURL(B16)&amp;"&amp;admision="&amp;ENCODEURL(C16&amp;" persona"&amp;IF(C16=1,"","s"))&amp;IF(D16&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D16),""))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="F17" s="2">
-        <f>IF(B17="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A17)&amp;"&amp;invitado="&amp;ENCODEURL(B17)&amp;IF(C17&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C17),"")&amp;"&amp;admision="&amp;ENCODEURL(D17&amp;" persona"&amp;IF(D17=1,"","s"))&amp;IF(E17&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E17),""))</f>
+      <c r="E17" s="2">
+        <f>IF(B17="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A17)&amp;"&amp;invitado="&amp;ENCODEURL(B17)&amp;"&amp;admision="&amp;ENCODEURL(C17&amp;" persona"&amp;IF(C17=1,"","s"))&amp;IF(D17&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D17),""))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="F18" s="2">
-        <f>IF(B18="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A18)&amp;"&amp;invitado="&amp;ENCODEURL(B18)&amp;IF(C18&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C18),"")&amp;"&amp;admision="&amp;ENCODEURL(D18&amp;" persona"&amp;IF(D18=1,"","s"))&amp;IF(E18&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E18),""))</f>
+      <c r="E18" s="2">
+        <f>IF(B18="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A18)&amp;"&amp;invitado="&amp;ENCODEURL(B18)&amp;"&amp;admision="&amp;ENCODEURL(C18&amp;" persona"&amp;IF(C18=1,"","s"))&amp;IF(D18&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D18),""))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="F19" s="2">
-        <f>IF(B19="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A19)&amp;"&amp;invitado="&amp;ENCODEURL(B19)&amp;IF(C19&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C19),"")&amp;"&amp;admision="&amp;ENCODEURL(D19&amp;" persona"&amp;IF(D19=1,"","s"))&amp;IF(E19&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E19),""))</f>
+      <c r="E19" s="2">
+        <f>IF(B19="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A19)&amp;"&amp;invitado="&amp;ENCODEURL(B19)&amp;"&amp;admision="&amp;ENCODEURL(C19&amp;" persona"&amp;IF(C19=1,"","s"))&amp;IF(D19&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D19),""))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="F20" s="2">
-        <f>IF(B20="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A20)&amp;"&amp;invitado="&amp;ENCODEURL(B20)&amp;IF(C20&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C20),"")&amp;"&amp;admision="&amp;ENCODEURL(D20&amp;" persona"&amp;IF(D20=1,"","s"))&amp;IF(E20&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E20),""))</f>
+      <c r="E20" s="2">
+        <f>IF(B20="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A20)&amp;"&amp;invitado="&amp;ENCODEURL(B20)&amp;"&amp;admision="&amp;ENCODEURL(C20&amp;" persona"&amp;IF(C20=1,"","s"))&amp;IF(D20&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D20),""))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="F21" s="2">
-        <f>IF(B21="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A21)&amp;"&amp;invitado="&amp;ENCODEURL(B21)&amp;IF(C21&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C21),"")&amp;"&amp;admision="&amp;ENCODEURL(D21&amp;" persona"&amp;IF(D21=1,"","s"))&amp;IF(E21&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E21),""))</f>
+      <c r="E21" s="2">
+        <f>IF(B21="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A21)&amp;"&amp;invitado="&amp;ENCODEURL(B21)&amp;"&amp;admision="&amp;ENCODEURL(C21&amp;" persona"&amp;IF(C21=1,"","s"))&amp;IF(D21&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D21),""))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="F22" s="2">
-        <f>IF(B22="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A22)&amp;"&amp;invitado="&amp;ENCODEURL(B22)&amp;IF(C22&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C22),"")&amp;"&amp;admision="&amp;ENCODEURL(D22&amp;" persona"&amp;IF(D22=1,"","s"))&amp;IF(E22&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E22),""))</f>
+      <c r="E22" s="2">
+        <f>IF(B22="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A22)&amp;"&amp;invitado="&amp;ENCODEURL(B22)&amp;"&amp;admision="&amp;ENCODEURL(C22&amp;" persona"&amp;IF(C22=1,"","s"))&amp;IF(D22&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D22),""))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="F23" s="2">
-        <f>IF(B23="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A23)&amp;"&amp;invitado="&amp;ENCODEURL(B23)&amp;IF(C23&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C23),"")&amp;"&amp;admision="&amp;ENCODEURL(D23&amp;" persona"&amp;IF(D23=1,"","s"))&amp;IF(E23&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E23),""))</f>
+      <c r="E23" s="2">
+        <f>IF(B23="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A23)&amp;"&amp;invitado="&amp;ENCODEURL(B23)&amp;"&amp;admision="&amp;ENCODEURL(C23&amp;" persona"&amp;IF(C23=1,"","s"))&amp;IF(D23&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D23),""))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="F24" s="2">
-        <f>IF(B24="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A24)&amp;"&amp;invitado="&amp;ENCODEURL(B24)&amp;IF(C24&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C24),"")&amp;"&amp;admision="&amp;ENCODEURL(D24&amp;" persona"&amp;IF(D24=1,"","s"))&amp;IF(E24&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E24),""))</f>
+      <c r="E24" s="2">
+        <f>IF(B24="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A24)&amp;"&amp;invitado="&amp;ENCODEURL(B24)&amp;"&amp;admision="&amp;ENCODEURL(C24&amp;" persona"&amp;IF(C24=1,"","s"))&amp;IF(D24&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D24),""))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="F25" s="2">
-        <f>IF(B25="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A25)&amp;"&amp;invitado="&amp;ENCODEURL(B25)&amp;IF(C25&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C25),"")&amp;"&amp;admision="&amp;ENCODEURL(D25&amp;" persona"&amp;IF(D25=1,"","s"))&amp;IF(E25&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E25),""))</f>
+      <c r="E25" s="2">
+        <f>IF(B25="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A25)&amp;"&amp;invitado="&amp;ENCODEURL(B25)&amp;"&amp;admision="&amp;ENCODEURL(C25&amp;" persona"&amp;IF(C25=1,"","s"))&amp;IF(D25&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D25),""))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="F26" s="2">
-        <f>IF(B26="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A26)&amp;"&amp;invitado="&amp;ENCODEURL(B26)&amp;IF(C26&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C26),"")&amp;"&amp;admision="&amp;ENCODEURL(D26&amp;" persona"&amp;IF(D26=1,"","s"))&amp;IF(E26&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E26),""))</f>
+      <c r="E26" s="2">
+        <f>IF(B26="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A26)&amp;"&amp;invitado="&amp;ENCODEURL(B26)&amp;"&amp;admision="&amp;ENCODEURL(C26&amp;" persona"&amp;IF(C26=1,"","s"))&amp;IF(D26&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D26),""))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="F27" s="2">
-        <f>IF(B27="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A27)&amp;"&amp;invitado="&amp;ENCODEURL(B27)&amp;IF(C27&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C27),"")&amp;"&amp;admision="&amp;ENCODEURL(D27&amp;" persona"&amp;IF(D27=1,"","s"))&amp;IF(E27&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E27),""))</f>
+      <c r="E27" s="2">
+        <f>IF(B27="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A27)&amp;"&amp;invitado="&amp;ENCODEURL(B27)&amp;"&amp;admision="&amp;ENCODEURL(C27&amp;" persona"&amp;IF(C27=1,"","s"))&amp;IF(D27&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D27),""))</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="F28" s="2">
-        <f>IF(B28="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A28)&amp;"&amp;invitado="&amp;ENCODEURL(B28)&amp;IF(C28&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C28),"")&amp;"&amp;admision="&amp;ENCODEURL(D28&amp;" persona"&amp;IF(D28=1,"","s"))&amp;IF(E28&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E28),""))</f>
+      <c r="E28" s="2">
+        <f>IF(B28="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A28)&amp;"&amp;invitado="&amp;ENCODEURL(B28)&amp;"&amp;admision="&amp;ENCODEURL(C28&amp;" persona"&amp;IF(C28=1,"","s"))&amp;IF(D28&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D28),""))</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="F29" s="2">
-        <f>IF(B29="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A29)&amp;"&amp;invitado="&amp;ENCODEURL(B29)&amp;IF(C29&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C29),"")&amp;"&amp;admision="&amp;ENCODEURL(D29&amp;" persona"&amp;IF(D29=1,"","s"))&amp;IF(E29&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E29),""))</f>
+      <c r="E29" s="2">
+        <f>IF(B29="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A29)&amp;"&amp;invitado="&amp;ENCODEURL(B29)&amp;"&amp;admision="&amp;ENCODEURL(C29&amp;" persona"&amp;IF(C29=1,"","s"))&amp;IF(D29&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D29),""))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="F30" s="2">
-        <f>IF(B30="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A30)&amp;"&amp;invitado="&amp;ENCODEURL(B30)&amp;IF(C30&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C30),"")&amp;"&amp;admision="&amp;ENCODEURL(D30&amp;" persona"&amp;IF(D30=1,"","s"))&amp;IF(E30&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E30),""))</f>
+      <c r="E30" s="2">
+        <f>IF(B30="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A30)&amp;"&amp;invitado="&amp;ENCODEURL(B30)&amp;"&amp;admision="&amp;ENCODEURL(C30&amp;" persona"&amp;IF(C30=1,"","s"))&amp;IF(D30&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D30),""))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="F31" s="2">
-        <f>IF(B31="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A31)&amp;"&amp;invitado="&amp;ENCODEURL(B31)&amp;IF(C31&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C31),"")&amp;"&amp;admision="&amp;ENCODEURL(D31&amp;" persona"&amp;IF(D31=1,"","s"))&amp;IF(E31&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E31),""))</f>
+      <c r="E31" s="2">
+        <f>IF(B31="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A31)&amp;"&amp;invitado="&amp;ENCODEURL(B31)&amp;"&amp;admision="&amp;ENCODEURL(C31&amp;" persona"&amp;IF(C31=1,"","s"))&amp;IF(D31&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D31),""))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="F32" s="2">
-        <f>IF(B32="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A32)&amp;"&amp;invitado="&amp;ENCODEURL(B32)&amp;IF(C32&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C32),"")&amp;"&amp;admision="&amp;ENCODEURL(D32&amp;" persona"&amp;IF(D32=1,"","s"))&amp;IF(E32&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E32),""))</f>
+      <c r="E32" s="2">
+        <f>IF(B32="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A32)&amp;"&amp;invitado="&amp;ENCODEURL(B32)&amp;"&amp;admision="&amp;ENCODEURL(C32&amp;" persona"&amp;IF(C32=1,"","s"))&amp;IF(D32&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D32),""))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="F33" s="2">
-        <f>IF(B33="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A33)&amp;"&amp;invitado="&amp;ENCODEURL(B33)&amp;IF(C33&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C33),"")&amp;"&amp;admision="&amp;ENCODEURL(D33&amp;" persona"&amp;IF(D33=1,"","s"))&amp;IF(E33&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E33),""))</f>
+      <c r="E33" s="2">
+        <f>IF(B33="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A33)&amp;"&amp;invitado="&amp;ENCODEURL(B33)&amp;"&amp;admision="&amp;ENCODEURL(C33&amp;" persona"&amp;IF(C33=1,"","s"))&amp;IF(D33&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D33),""))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="F34" s="2">
-        <f>IF(B34="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A34)&amp;"&amp;invitado="&amp;ENCODEURL(B34)&amp;IF(C34&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C34),"")&amp;"&amp;admision="&amp;ENCODEURL(D34&amp;" persona"&amp;IF(D34=1,"","s"))&amp;IF(E34&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E34),""))</f>
+      <c r="E34" s="2">
+        <f>IF(B34="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A34)&amp;"&amp;invitado="&amp;ENCODEURL(B34)&amp;"&amp;admision="&amp;ENCODEURL(C34&amp;" persona"&amp;IF(C34=1,"","s"))&amp;IF(D34&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D34),""))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="F35" s="2">
-        <f>IF(B35="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A35)&amp;"&amp;invitado="&amp;ENCODEURL(B35)&amp;IF(C35&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C35),"")&amp;"&amp;admision="&amp;ENCODEURL(D35&amp;" persona"&amp;IF(D35=1,"","s"))&amp;IF(E35&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E35),""))</f>
+      <c r="E35" s="2">
+        <f>IF(B35="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A35)&amp;"&amp;invitado="&amp;ENCODEURL(B35)&amp;"&amp;admision="&amp;ENCODEURL(C35&amp;" persona"&amp;IF(C35=1,"","s"))&amp;IF(D35&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D35),""))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="F36" s="2">
-        <f>IF(B36="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A36)&amp;"&amp;invitado="&amp;ENCODEURL(B36)&amp;IF(C36&lt;&gt;"","&amp;firma="&amp;ENCODEURL(C36),"")&amp;"&amp;admision="&amp;ENCODEURL(D36&amp;" persona"&amp;IF(D36=1,"","s"))&amp;IF(E36&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(E36),""))</f>
+      <c r="E36" s="2">
+        <f>IF(B36="","",$B$1&amp;"?titulo="&amp;ENCODEURL(A36)&amp;"&amp;invitado="&amp;ENCODEURL(B36)&amp;"&amp;admision="&amp;ENCODEURL(C36&amp;" persona"&amp;IF(C36=1,"","s"))&amp;IF(D36&lt;&gt;"","&amp;invitados="&amp;ENCODEURL(D36),""))</f>
         <v/>
       </c>
     </row>
@@ -813,65 +796,61 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>4. Columna 'Firma / nota': opcional, aparece como nota personalizada.</t>
+          <t>4. Columna 'Cupos (número)': cuántas personas puede confirmar esa invitación (ej. 1, 2, 3...).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>5. Columna 'Cupos (número)': cuántas personas puede confirmar esa invitación (ej. 1, 2, 3...).</t>
+          <t>5. Columna 'Invitados (nombres...)': SOLO si quieres que en el formulario aparezca una lista para marcar</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>6. Columna 'Invitados (nombres...)': SOLO si quieres que en el formulario aparezca una lista para marcar</t>
+          <t xml:space="preserve">   quién sí asiste, por nombre. Escribe los nombres separados por coma, ej:</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   quién sí asiste, por nombre. Escribe los nombres separados por coma, ej:</t>
+          <t xml:space="preserve">   Adela Parrales, Juan Parrales, María Parrales</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Adela Parrales, Juan Parrales, María Parrales</t>
+          <t xml:space="preserve">   Si la dejas vacía, el formulario mostrará solo un selector numérico (1, 2, 3 personas...).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Si la dejas vacía, el formulario mostrará solo un selector numérico (1, 2, 3 personas...).</t>
+          <t xml:space="preserve">   El número de nombres debe coincidir con los 'Cupos'.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   El número de nombres debe coincidir con los 'Cupos'.</t>
+          <t>6. La columna 'URL generada' se arma sola con una fórmula. Cópiala y envíasela a cada invitado</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>7. La columna 'URL generada' se arma sola con una fórmula. Cópiala y envíasela a cada invitado</t>
+          <t xml:space="preserve">   (por WhatsApp, mensaje de texto, etc.).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   (por WhatsApp, mensaje de texto, etc.).</t>
-        </is>
-      </c>
+      <c r="A14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr"/>

</xml_diff>